<commit_message>
BRD-03, BRD-04 and BRD-11 v2.1: FRS and UX screen documents rebuilt on the retaken document images
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-04_Collections/08_BIBS_UXScreens_BRD-04_Collections_v2.1.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-04_Collections/08_BIBS_UXScreens_BRD-04_Collections_v2.1.xlsx
@@ -6184,7 +6184,7 @@
       </c>
       <c r="K81" s="45" t="inlineStr">
         <is>
-          <t>Outstanding PR List: first page as generated</t>
+          <t>Outstanding PR List: first page as generated: the report header and a selection of the columns</t>
         </is>
       </c>
       <c r="L81" s="45" t="inlineStr">
@@ -6244,7 +6244,7 @@
       </c>
       <c r="K82" s="45" t="inlineStr">
         <is>
-          <t>Full Production Report: first page as generated</t>
+          <t>Full Production Report: first page as generated: the report header and a selection of the columns</t>
         </is>
       </c>
       <c r="L82" s="45" t="inlineStr">
@@ -6304,7 +6304,7 @@
       </c>
       <c r="K83" s="45" t="inlineStr">
         <is>
-          <t>DP PR for Reversal and PR 2307 for Reversal files: first page as generated</t>
+          <t>DP PR for Reversal and PR 2307 for Reversal files: first page as generated: the report header and a selection of the columns</t>
         </is>
       </c>
       <c r="L83" s="45" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="K84" s="45" t="inlineStr">
         <is>
-          <t>For Application To Invoice file: first page as generated</t>
+          <t>For Application To Invoice file: the file as generated, shown field by field (its first line names the fields)</t>
         </is>
       </c>
       <c r="L84" s="45" t="inlineStr">

</xml_diff>